<commit_message>
added note in weather input columns
</commit_message>
<xml_diff>
--- a/FSP_Wheat/FSP_Excel_Input_WH_NT_2025_test.xlsx
+++ b/FSP_Wheat/FSP_Excel_Input_WH_NT_2025_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\WheatSim_GUI\FSP_Wheat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08127B8-476C-49B0-9C4B-FA7EA6C287B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F872AC1-570F-4A9E-8360-667763733EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27360" yWindow="5985" windowWidth="26160" windowHeight="10965" tabRatio="860" xr2:uid="{DF0A0CE0-D649-4449-A8FD-3001850BE46E}"/>
+    <workbookView xWindow="-27360" yWindow="10590" windowWidth="26160" windowHeight="6360" tabRatio="860" activeTab="2" xr2:uid="{DF0A0CE0-D649-4449-A8FD-3001850BE46E}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="2" r:id="rId1"/>
@@ -93,6 +93,65 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={E4936F07-87CF-40A5-9C99-A16743B24F1F}</author>
+    <author>tc={86D6701B-FB3C-454B-8A85-63F7D87999B1}</author>
+    <author>tc={DEC47F63-DC74-4E21-B97E-879D976DAB27}</author>
+    <author>tc={2F9C332F-ACC1-4A9F-8071-344C3CD7307E}</author>
+    <author>tc={D1F24C2E-CFE1-4FE0-813B-470E0B695375}</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{E4936F07-87CF-40A5-9C99-A16743B24F1F}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    daily concentration of N in rainfall
+</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="1" shapeId="0" xr:uid="{86D6701B-FB3C-454B-8A85-63F7D87999B1}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+     #If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="2" shapeId="0" xr:uid="{DEC47F63-DC74-4E21-B97E-879D976DAB27}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    #If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="3" shapeId="0" xr:uid="{2F9C332F-ACC1-4A9F-8071-344C3CD7307E}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    #If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="4" shapeId="0" xr:uid="{D1F24C2E-CFE1-4FE0-813B-470E0B695375}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    #If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
     <author>tc={2FBD78F9-86E2-443E-A3F3-9DF369530A73}</author>
     <author>tc={2AFAD96D-4597-4C2E-B26C-3696E048E29F}</author>
     <author>tc={1EB72D7A-C7BF-46D4-9A9A-2E7E9CC7D386}</author>
@@ -167,7 +226,7 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
@@ -278,7 +337,7 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
@@ -379,7 +438,7 @@
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
@@ -480,7 +539,7 @@
 </comments>
 </file>
 
-<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={9CD0834F-37B7-4414-967F-1A3C38607D83}</author>
@@ -1548,7 +1607,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1664,6 +1723,12 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="14">
@@ -14497,6 +14562,31 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="H1" dT="2026-05-27T19:20:24.41" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{E4936F07-87CF-40A5-9C99-A16743B24F1F}">
+    <text xml:space="preserve">daily concentration of N in rainfall
+</text>
+  </threadedComment>
+  <threadedComment ref="R1" dT="2026-05-27T19:20:55.80" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{86D6701B-FB3C-454B-8A85-63F7D87999B1}">
+    <text xml:space="preserve"> #If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</text>
+  </threadedComment>
+  <threadedComment ref="S1" dT="2026-05-27T19:21:06.51" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{DEC47F63-DC74-4E21-B97E-879D976DAB27}">
+    <text xml:space="preserve">#If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</text>
+  </threadedComment>
+  <threadedComment ref="T1" dT="2026-05-27T19:20:45.66" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{2F9C332F-ACC1-4A9F-8071-344C3CD7307E}">
+    <text xml:space="preserve">#If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</text>
+  </threadedComment>
+  <threadedComment ref="V1" dT="2026-05-27T19:21:18.77" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{D1F24C2E-CFE1-4FE0-813B-470E0B695375}">
+    <text xml:space="preserve">#If, wind, rainIntensity, dailyConc or CO2 are 0 then the averages must be input. 
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B1" dT="2023-03-28T19:20:39.32" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{2FBD78F9-86E2-443E-A3F3-9DF369530A73}">
     <text>EJ:Initialtime</text>
   </threadedComment>
@@ -14526,7 +14616,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="G1" dT="2023-06-07T16:35:10.98" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{CB550BE2-26D9-4EE1-90D1-6D4DC9225BBA}">
     <text>EJ: sowing date should be later than EndDate in Time tab</text>
@@ -14541,7 +14631,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment5.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="F2" dT="2024-09-12T21:33:11.56" personId="{080D0DFC-C7D2-484C-9C84-E180B7FC9FD1}" id="{9CD0834F-37B7-4414-967F-1A3C38607D83}">
     <text>Dennis's ponding irrigation</text>
@@ -32325,7 +32415,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDD7FD97-5EA5-4DA5-ACDD-C1B0B0E3B3BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDD7FD97-5EA5-4DA5-ACDD-C1B0B0E3B3BD}">
   <sheetPr codeName="Sheet18"/>
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -32499,6 +32589,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
added note to the weather column
</commit_message>
<xml_diff>
--- a/FSP_Wheat/FSP_Excel_Input_WH_NT_2025_test.xlsx
+++ b/FSP_Wheat/FSP_Excel_Input_WH_NT_2025_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\WheatSim_GUI\FSP_Wheat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F872AC1-570F-4A9E-8360-667763733EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82E79E7-0B26-4184-A6C9-7EFE8FB3A180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27360" yWindow="10590" windowWidth="26160" windowHeight="6360" tabRatio="860" activeTab="2" xr2:uid="{DF0A0CE0-D649-4449-A8FD-3001850BE46E}"/>
+    <workbookView xWindow="-27360" yWindow="8220" windowWidth="26160" windowHeight="8730" tabRatio="860" activeTab="6" xr2:uid="{DF0A0CE0-D649-4449-A8FD-3001850BE46E}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="2" r:id="rId1"/>
@@ -39498,6 +39498,19 @@
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>